<commit_message>
Major Update: Structural PDF Extraction, Multi-item Accumulation, and Global Batch Mapping
</commit_message>
<xml_diff>
--- a/MONITORING PK-PM 31 PUPUK 2026.xlsx
+++ b/MONITORING PK-PM 31 PUPUK 2026.xlsx
@@ -76,7 +76,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -168,6 +168,15 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3649,15 +3658,20 @@
       <c r="M2" s="31" t="n">
         <v>217503000</v>
       </c>
-      <c r="N2" s="16" t="n"/>
-      <c r="O2" s="16" t="n"/>
+      <c r="N2" s="38" t="n">
+        <v>6591000</v>
+      </c>
+      <c r="O2" s="39" t="n">
+        <v>1977300000</v>
+      </c>
       <c r="T2" s="36">
         <f>O2+Q2+S2</f>
         <v/>
       </c>
-      <c r="U2" s="35">
-        <f>K2-T2</f>
-        <v/>
+      <c r="U2" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3705,15 +3719,20 @@
       <c r="M3" s="31" t="n">
         <v>2530000</v>
       </c>
-      <c r="R3" s="16" t="n"/>
-      <c r="S3" s="16" t="n"/>
+      <c r="R3" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S3" s="39" t="n">
+        <v>23000000</v>
+      </c>
       <c r="T3" s="36">
         <f>O3+Q3+S3</f>
         <v/>
       </c>
-      <c r="U3" s="35">
-        <f>K3-T3</f>
-        <v/>
+      <c r="U3" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3761,15 +3780,20 @@
       <c r="M4" s="31" t="n">
         <v>2403500</v>
       </c>
-      <c r="R4" s="16" t="n"/>
-      <c r="S4" s="16" t="n"/>
+      <c r="R4" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S4" s="39" t="n">
+        <v>21850000</v>
+      </c>
       <c r="T4" s="36">
         <f>O4+Q4+S4</f>
         <v/>
       </c>
-      <c r="U4" s="35">
-        <f>K4-T4</f>
-        <v/>
+      <c r="U4" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3817,15 +3841,20 @@
       <c r="M5" s="31" t="n">
         <v>570900</v>
       </c>
-      <c r="R5" s="16" t="n"/>
-      <c r="S5" s="16" t="n"/>
+      <c r="R5" s="38" t="n">
+        <v>173</v>
+      </c>
+      <c r="S5" s="39" t="n">
+        <v>5190000</v>
+      </c>
       <c r="T5" s="36">
         <f>O5+Q5+S5</f>
         <v/>
       </c>
-      <c r="U5" s="35">
-        <f>K5-T5</f>
-        <v/>
+      <c r="U5" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3873,15 +3902,20 @@
       <c r="M6" s="31" t="n">
         <v>14219865</v>
       </c>
-      <c r="R6" s="16" t="n"/>
-      <c r="S6" s="16" t="n"/>
+      <c r="R6" s="38" t="n">
+        <v>3450</v>
+      </c>
+      <c r="S6" s="39" t="n">
+        <v>129271500</v>
+      </c>
       <c r="T6" s="36">
         <f>O6+Q6+S6</f>
         <v/>
       </c>
-      <c r="U6" s="35">
-        <f>K6-T6</f>
-        <v/>
+      <c r="U6" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -3934,15 +3968,20 @@
       <c r="M7" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N7" s="16" t="n"/>
-      <c r="O7" s="16" t="n"/>
+      <c r="N7" s="38" t="n">
+        <v>6591000</v>
+      </c>
+      <c r="O7" s="39" t="n">
+        <v>1318200000</v>
+      </c>
       <c r="T7" s="36">
         <f>O7+Q7+S7</f>
         <v/>
       </c>
-      <c r="U7" s="35">
-        <f>K7-T7</f>
-        <v/>
+      <c r="U7" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8" hidden="1">
@@ -4055,15 +4094,20 @@
       <c r="M9" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N9" s="16" t="n"/>
-      <c r="O9" s="13" t="n"/>
+      <c r="N9" s="38" t="n">
+        <v>6591000</v>
+      </c>
+      <c r="O9" s="13" t="n">
+        <v>1318200000</v>
+      </c>
       <c r="T9" s="36">
         <f>O9+Q9+S9</f>
         <v/>
       </c>
-      <c r="U9" s="35">
-        <f>K9-T9</f>
-        <v/>
+      <c r="U9" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -4111,15 +4155,20 @@
       <c r="M10" s="31" t="n">
         <v>4680500</v>
       </c>
-      <c r="R10" s="16" t="n"/>
-      <c r="S10" s="13" t="n"/>
+      <c r="R10" s="38" t="n">
+        <v>1150</v>
+      </c>
+      <c r="S10" s="13" t="n">
+        <v>42550000</v>
+      </c>
       <c r="T10" s="36">
         <f>O10+Q10+S10</f>
         <v/>
       </c>
-      <c r="U10" s="35">
-        <f>K10-T10</f>
-        <v/>
+      <c r="U10" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -4167,15 +4216,20 @@
       <c r="M11" s="31" t="n">
         <v>12650000</v>
       </c>
-      <c r="R11" s="16" t="n"/>
-      <c r="S11" s="13" t="n"/>
+      <c r="R11" s="38" t="n">
+        <v>2875</v>
+      </c>
+      <c r="S11" s="13" t="n">
+        <v>115000000</v>
+      </c>
       <c r="T11" s="36">
         <f>O11+Q11+S11</f>
         <v/>
       </c>
-      <c r="U11" s="35">
-        <f>K11-T11</f>
-        <v/>
+      <c r="U11" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -4223,15 +4277,20 @@
       <c r="M12" s="31" t="n">
         <v>9297750</v>
       </c>
-      <c r="R12" s="16" t="n"/>
-      <c r="S12" s="13" t="n"/>
+      <c r="R12" s="38" t="n">
+        <v>2300</v>
+      </c>
+      <c r="S12" s="13" t="n">
+        <v>84525000</v>
+      </c>
       <c r="T12" s="36">
         <f>O12+Q12+S12</f>
         <v/>
       </c>
-      <c r="U12" s="35">
-        <f>K12-T12</f>
-        <v/>
+      <c r="U12" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -4283,6 +4342,12 @@
       </c>
       <c r="M13" s="31" t="n">
         <v>18150000</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>550</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>165000000</v>
       </c>
       <c r="R13" s="16" t="n"/>
       <c r="S13" s="13" t="n"/>
@@ -4290,9 +4355,10 @@
         <f>O13+Q13+S13</f>
         <v/>
       </c>
-      <c r="U13" s="35">
-        <f>K13-T13</f>
-        <v/>
+      <c r="U13" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -4340,15 +4406,20 @@
       <c r="M14" s="31" t="n">
         <v>8855000</v>
       </c>
-      <c r="R14" s="16" t="n"/>
-      <c r="S14" s="13" t="n"/>
+      <c r="R14" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S14" s="13" t="n">
+        <v>80500000</v>
+      </c>
       <c r="T14" s="36">
         <f>O14+Q14+S14</f>
         <v/>
       </c>
-      <c r="U14" s="35">
-        <f>K14-T14</f>
-        <v/>
+      <c r="U14" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -4401,15 +4472,20 @@
       <c r="M15" s="31" t="n">
         <v>77858000</v>
       </c>
-      <c r="N15" s="16" t="n"/>
-      <c r="O15" s="13" t="n"/>
+      <c r="N15" s="38" t="n">
+        <v>7078000</v>
+      </c>
+      <c r="O15" s="13" t="n">
+        <v>707800000</v>
+      </c>
       <c r="T15" s="36">
         <f>O15+Q15+S15</f>
         <v/>
       </c>
-      <c r="U15" s="35">
-        <f>K15-T15</f>
-        <v/>
+      <c r="U15" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -4462,15 +4538,20 @@
       <c r="M16" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N16" s="16" t="n"/>
-      <c r="O16" s="13" t="n"/>
+      <c r="N16" s="38" t="n">
+        <v>6591000</v>
+      </c>
+      <c r="O16" s="13" t="n">
+        <v>1318200000</v>
+      </c>
       <c r="T16" s="36">
         <f>O16+Q16+S16</f>
         <v/>
       </c>
-      <c r="U16" s="35">
-        <f>K16-T16</f>
-        <v/>
+      <c r="U16" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -4523,15 +4604,20 @@
       <c r="M17" s="31" t="n">
         <v>1960750</v>
       </c>
-      <c r="R17" s="16" t="n"/>
-      <c r="S17" s="16" t="n"/>
+      <c r="R17" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S17" s="39" t="n">
+        <v>17825000</v>
+      </c>
       <c r="T17" s="36">
         <f>O17+Q17+S17</f>
         <v/>
       </c>
-      <c r="U17" s="35">
-        <f>K17-T17</f>
-        <v/>
+      <c r="U17" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -4584,15 +4670,20 @@
       <c r="M18" s="31" t="n">
         <v>3921500</v>
       </c>
-      <c r="R18" s="16" t="n"/>
-      <c r="S18" s="16" t="n"/>
+      <c r="R18" s="38" t="n">
+        <v>1150</v>
+      </c>
+      <c r="S18" s="39" t="n">
+        <v>35650000</v>
+      </c>
       <c r="T18" s="36">
         <f>O18+Q18+S18</f>
         <v/>
       </c>
-      <c r="U18" s="35">
-        <f>K18-T18</f>
-        <v/>
+      <c r="U18" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -4640,15 +4731,20 @@
       <c r="M19" s="31" t="n">
         <v>13768480</v>
       </c>
-      <c r="R19" s="16" t="n"/>
-      <c r="S19" s="16" t="n"/>
+      <c r="R19" s="38" t="n">
+        <v>160</v>
+      </c>
+      <c r="S19" s="39" t="n">
+        <v>125168000</v>
+      </c>
       <c r="T19" s="36">
         <f>O19+Q19+S19</f>
         <v/>
       </c>
-      <c r="U19" s="35">
-        <f>K19-T19</f>
-        <v/>
+      <c r="U19" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -4701,15 +4797,20 @@
       <c r="M20" s="31" t="n">
         <v>2277000</v>
       </c>
-      <c r="R20" s="16" t="n"/>
-      <c r="S20" s="16" t="n"/>
+      <c r="R20" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S20" s="39" t="n">
+        <v>20700000</v>
+      </c>
       <c r="T20" s="36">
         <f>O20+Q20+S20</f>
         <v/>
       </c>
-      <c r="U20" s="35">
-        <f>K20-T20</f>
-        <v/>
+      <c r="U20" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -4831,15 +4932,20 @@
       <c r="O22" s="16" t="n"/>
       <c r="P22" s="16" t="n"/>
       <c r="Q22" s="16" t="n"/>
-      <c r="R22" s="16" t="n"/>
-      <c r="S22" s="16" t="n"/>
+      <c r="R22" s="38" t="n">
+        <v>170</v>
+      </c>
+      <c r="S22" s="39" t="n">
+        <v>5100000</v>
+      </c>
       <c r="T22" s="36">
         <f>O22+Q22+S22</f>
         <v/>
       </c>
-      <c r="U22" s="35">
-        <f>K22-T22</f>
-        <v/>
+      <c r="U22" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -4896,15 +5002,20 @@
       <c r="O23" s="16" t="n"/>
       <c r="P23" s="16" t="n"/>
       <c r="Q23" s="16" t="n"/>
-      <c r="R23" s="16" t="n"/>
-      <c r="S23" s="18" t="n"/>
+      <c r="R23" s="38" t="n">
+        <v>580</v>
+      </c>
+      <c r="S23" s="18" t="n">
+        <v>104259640</v>
+      </c>
       <c r="T23" s="36">
         <f>O23+Q23+S23</f>
         <v/>
       </c>
-      <c r="U23" s="35">
-        <f>K23-T23</f>
-        <v/>
+      <c r="U23" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -4961,15 +5072,20 @@
       <c r="O24" s="16" t="n"/>
       <c r="P24" s="16" t="n"/>
       <c r="Q24" s="16" t="n"/>
-      <c r="R24" s="16" t="n"/>
-      <c r="S24" s="18" t="n"/>
+      <c r="R24" s="38" t="n">
+        <v>575</v>
+      </c>
+      <c r="S24" s="18" t="n">
+        <v>15525000</v>
+      </c>
       <c r="T24" s="36">
         <f>O24+Q24+S24</f>
         <v/>
       </c>
-      <c r="U24" s="35">
-        <f>K24-T24</f>
-        <v/>
+      <c r="U24" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -5017,15 +5133,20 @@
       <c r="M25" s="31" t="n">
         <v>2332000</v>
       </c>
-      <c r="R25" s="16" t="n"/>
-      <c r="S25" s="16" t="n"/>
+      <c r="R25" s="38" t="n">
+        <v>530</v>
+      </c>
+      <c r="S25" s="39" t="n">
+        <v>21200000</v>
+      </c>
       <c r="T25" s="36">
         <f>O25+Q25+S25</f>
         <v/>
       </c>
-      <c r="U25" s="35">
-        <f>K25-T25</f>
-        <v/>
+      <c r="U25" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -5073,15 +5194,20 @@
       <c r="M26" s="31" t="n">
         <v>3520000</v>
       </c>
-      <c r="R26" s="16" t="n"/>
-      <c r="S26" s="16" t="n"/>
+      <c r="R26" s="38" t="n">
+        <v>800</v>
+      </c>
+      <c r="S26" s="39" t="n">
+        <v>32000000</v>
+      </c>
       <c r="T26" s="36">
         <f>O26+Q26+S26</f>
         <v/>
       </c>
-      <c r="U26" s="35">
-        <f>K26-T26</f>
-        <v/>
+      <c r="U26" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -5129,15 +5255,20 @@
       <c r="M27" s="31" t="n">
         <v>704000</v>
       </c>
-      <c r="R27" s="16" t="n"/>
-      <c r="S27" s="16" t="n"/>
+      <c r="R27" s="38" t="n">
+        <v>160</v>
+      </c>
+      <c r="S27" s="39" t="n">
+        <v>6400000</v>
+      </c>
       <c r="T27" s="36">
         <f>O27+Q27+S27</f>
         <v/>
       </c>
-      <c r="U27" s="35">
-        <f>K27-T27</f>
-        <v/>
+      <c r="U27" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -5190,8 +5321,12 @@
       <c r="M28" s="31" t="n">
         <v>696963960</v>
       </c>
-      <c r="N28" s="16" t="n"/>
-      <c r="O28" s="16" t="n"/>
+      <c r="N28" s="38" t="n">
+        <v>6426000</v>
+      </c>
+      <c r="O28" s="39" t="n">
+        <v>6336036000</v>
+      </c>
       <c r="P28" s="16" t="n"/>
       <c r="Q28" s="16" t="n"/>
       <c r="R28" s="16" t="n"/>
@@ -5200,9 +5335,10 @@
         <f>O28+Q28+S28</f>
         <v/>
       </c>
-      <c r="U28" s="35">
-        <f>K28-T28</f>
-        <v/>
+      <c r="U28" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -5255,8 +5391,12 @@
       <c r="M29" s="31" t="n">
         <v>159043500</v>
       </c>
-      <c r="N29" s="16" t="n"/>
-      <c r="O29" s="13" t="n"/>
+      <c r="N29" s="38" t="n">
+        <v>6426000</v>
+      </c>
+      <c r="O29" s="13" t="n">
+        <v>1445850000</v>
+      </c>
       <c r="P29" s="16" t="n"/>
       <c r="Q29" s="16" t="n"/>
       <c r="R29" s="16" t="n"/>
@@ -5265,9 +5405,10 @@
         <f>O29+Q29+S29</f>
         <v/>
       </c>
-      <c r="U29" s="35">
-        <f>K29-T29</f>
-        <v/>
+      <c r="U29" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -5319,15 +5460,20 @@
       <c r="O30" s="16" t="n"/>
       <c r="P30" s="16" t="n"/>
       <c r="Q30" s="16" t="n"/>
-      <c r="R30" s="16" t="n"/>
-      <c r="S30" s="18" t="n"/>
+      <c r="R30" s="38" t="n">
+        <v>640</v>
+      </c>
+      <c r="S30" s="18" t="n">
+        <v>25600000</v>
+      </c>
       <c r="T30" s="36">
         <f>O30+Q30+S30</f>
         <v/>
       </c>
-      <c r="U30" s="35">
-        <f>K30-T30</f>
-        <v/>
+      <c r="U30" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -5380,8 +5526,12 @@
       <c r="M31" s="31" t="n">
         <v>473660000</v>
       </c>
-      <c r="N31" s="16" t="n"/>
-      <c r="O31" s="13" t="n"/>
+      <c r="N31" s="38" t="n">
+        <v>8612000</v>
+      </c>
+      <c r="O31" s="13" t="n">
+        <v>4306000000</v>
+      </c>
       <c r="P31" s="16" t="n"/>
       <c r="Q31" s="16" t="n"/>
       <c r="R31" s="16" t="n"/>
@@ -5390,9 +5540,10 @@
         <f>O31+Q31+S31</f>
         <v/>
       </c>
-      <c r="U31" s="35">
-        <f>K31-T31</f>
-        <v/>
+      <c r="U31" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -5500,15 +5651,20 @@
       <c r="M33" s="31" t="n">
         <v>1408000</v>
       </c>
-      <c r="R33" s="16" t="n"/>
-      <c r="S33" s="16" t="n"/>
+      <c r="R33" s="38" t="n">
+        <v>320</v>
+      </c>
+      <c r="S33" s="39" t="n">
+        <v>12800000</v>
+      </c>
       <c r="T33" s="36">
         <f>O33+Q33+S33</f>
         <v/>
       </c>
-      <c r="U33" s="35">
-        <f>K33-T33</f>
-        <v/>
+      <c r="U33" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -5556,15 +5712,20 @@
       <c r="M34" s="31" t="n">
         <v>1408000</v>
       </c>
-      <c r="R34" s="16" t="n"/>
-      <c r="S34" s="16" t="n"/>
+      <c r="R34" s="38" t="n">
+        <v>320</v>
+      </c>
+      <c r="S34" s="39" t="n">
+        <v>12800000</v>
+      </c>
       <c r="T34" s="36">
         <f>O34+Q34+S34</f>
         <v/>
       </c>
-      <c r="U34" s="35">
-        <f>K34-T34</f>
-        <v/>
+      <c r="U34" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -5612,15 +5773,20 @@
       <c r="M35" s="31" t="n">
         <v>2662000</v>
       </c>
-      <c r="R35" s="16" t="n"/>
-      <c r="S35" s="13" t="n"/>
+      <c r="R35" s="38" t="n">
+        <v>605</v>
+      </c>
+      <c r="S35" s="13" t="n">
+        <v>24200000</v>
+      </c>
       <c r="T35" s="36">
         <f>O35+Q35+S35</f>
         <v/>
       </c>
-      <c r="U35" s="35">
-        <f>K35-T35</f>
-        <v/>
+      <c r="U35" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -5668,15 +5834,20 @@
       <c r="M36" s="31" t="n">
         <v>91245000</v>
       </c>
-      <c r="N36" s="14" t="n"/>
-      <c r="O36" s="13" t="n"/>
+      <c r="N36" s="40" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O36" s="13" t="n">
+        <v>829500000</v>
+      </c>
       <c r="T36" s="36">
         <f>O36+Q36+S36</f>
         <v/>
       </c>
-      <c r="U36" s="35">
-        <f>K36-T36</f>
-        <v/>
+      <c r="U36" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -5724,15 +5895,20 @@
       <c r="M37" s="31" t="n">
         <v>94503750</v>
       </c>
-      <c r="N37" s="14" t="n"/>
-      <c r="O37" s="13" t="n"/>
+      <c r="N37" s="40" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O37" s="13" t="n">
+        <v>859125000</v>
+      </c>
       <c r="T37" s="36">
         <f>O37+Q37+S37</f>
         <v/>
       </c>
-      <c r="U37" s="35">
-        <f>K37-T37</f>
-        <v/>
+      <c r="U37" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -5780,15 +5956,20 @@
       <c r="M38" s="31" t="n">
         <v>2552000</v>
       </c>
-      <c r="R38" s="16" t="n"/>
-      <c r="S38" s="18" t="n"/>
+      <c r="R38" s="38" t="n">
+        <v>580</v>
+      </c>
+      <c r="S38" s="18" t="n">
+        <v>23200000</v>
+      </c>
       <c r="T38" s="36">
         <f>O38+Q38+S38</f>
         <v/>
       </c>
-      <c r="U38" s="35">
-        <f>K38-T38</f>
-        <v/>
+      <c r="U38" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -5836,15 +6017,20 @@
       <c r="M39" s="31" t="n">
         <v>2937297</v>
       </c>
-      <c r="R39" s="16" t="n"/>
-      <c r="S39" s="18" t="n"/>
+      <c r="R39" s="38" t="n">
+        <v>117117.12</v>
+      </c>
+      <c r="S39" s="18" t="n">
+        <v>26702703.36</v>
+      </c>
       <c r="T39" s="36">
         <f>O39+Q39+S39</f>
         <v/>
       </c>
-      <c r="U39" s="35">
-        <f>K39-T39</f>
-        <v/>
+      <c r="U39" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -5892,8 +6078,12 @@
       <c r="M40" s="31" t="n">
         <v>543125000</v>
       </c>
-      <c r="N40" s="16" t="n"/>
-      <c r="O40" s="16" t="n"/>
+      <c r="N40" s="38" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O40" s="39" t="n">
+        <v>4937500000</v>
+      </c>
       <c r="P40" s="16" t="n"/>
       <c r="Q40" s="16" t="n"/>
       <c r="R40" s="16" t="n"/>
@@ -5902,9 +6092,10 @@
         <f>O40+Q40+S40</f>
         <v/>
       </c>
-      <c r="U40" s="35">
-        <f>K40-T40</f>
-        <v/>
+      <c r="U40" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="41" hidden="1">
@@ -5972,15 +6163,20 @@
       <c r="M43" s="31" t="n">
         <v>2442000</v>
       </c>
-      <c r="R43" s="16" t="n"/>
-      <c r="S43" s="18" t="n"/>
+      <c r="R43" s="38" t="n">
+        <v>555</v>
+      </c>
+      <c r="S43" s="18" t="n">
+        <v>22200000</v>
+      </c>
       <c r="T43" s="36">
         <f>O43+Q43+S43</f>
         <v/>
       </c>
-      <c r="U43" s="35">
-        <f>K43-T43</f>
-        <v/>
+      <c r="U43" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -6028,15 +6224,20 @@
       <c r="M44" s="31" t="n">
         <v>3256000</v>
       </c>
-      <c r="R44" s="16" t="n"/>
-      <c r="S44" s="18" t="n"/>
+      <c r="R44" s="38" t="n">
+        <v>740</v>
+      </c>
+      <c r="S44" s="18" t="n">
+        <v>29600000</v>
+      </c>
       <c r="T44" s="36">
         <f>O44+Q44+S44</f>
         <v/>
       </c>
-      <c r="U44" s="35">
-        <f>K44-T44</f>
-        <v/>
+      <c r="U44" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -6084,15 +6285,20 @@
       <c r="M45" s="31" t="n">
         <v>814000</v>
       </c>
-      <c r="R45" s="16" t="n"/>
-      <c r="S45" s="18" t="n"/>
+      <c r="R45" s="38" t="n">
+        <v>185</v>
+      </c>
+      <c r="S45" s="18" t="n">
+        <v>7400000</v>
+      </c>
       <c r="T45" s="36">
         <f>O45+Q45+S45</f>
         <v/>
       </c>
-      <c r="U45" s="35">
-        <f>K45-T45</f>
-        <v/>
+      <c r="U45" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -6140,6 +6346,12 @@
       <c r="M46" s="31" t="n">
         <v>238975000</v>
       </c>
+      <c r="N46" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>2172500000</v>
+      </c>
       <c r="T46" s="36" t="n">
         <v>2172500000</v>
       </c>
@@ -6194,6 +6406,12 @@
       <c r="M47" s="31" t="n">
         <v>22811250</v>
       </c>
+      <c r="N47" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O47" s="4" t="n">
+        <v>207375000</v>
+      </c>
       <c r="T47" s="36" t="n">
         <v>207375000</v>
       </c>
@@ -6247,14 +6465,21 @@
       </c>
       <c r="M48" s="31" t="n">
         <v>41277500</v>
+      </c>
+      <c r="N48" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O48" s="4" t="n">
+        <v>375250000</v>
       </c>
       <c r="T48" s="36">
         <f>O48+Q48+S48</f>
         <v/>
       </c>
-      <c r="U48" s="35">
-        <f>K48-T48</f>
-        <v/>
+      <c r="U48" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -6302,6 +6527,12 @@
       <c r="M49" s="31" t="n">
         <v>41277500</v>
       </c>
+      <c r="N49" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O49" s="4" t="n">
+        <v>375250000</v>
+      </c>
       <c r="T49" s="36" t="n">
         <v>375250000</v>
       </c>
@@ -6355,14 +6586,21 @@
       </c>
       <c r="M50" s="31" t="n">
         <v>256355000</v>
+      </c>
+      <c r="N50" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O50" s="4" t="n">
+        <v>2330500000</v>
       </c>
       <c r="T50" s="36">
         <f>O50+Q50+S50</f>
         <v/>
       </c>
-      <c r="U50" s="35">
-        <f>K50-T50</f>
-        <v/>
+      <c r="U50" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -6409,14 +6647,21 @@
       </c>
       <c r="M51" s="31" t="n">
         <v>304150000</v>
+      </c>
+      <c r="N51" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O51" s="4" t="n">
+        <v>2765000000</v>
       </c>
       <c r="T51" s="36">
         <f>O51+Q51+S51</f>
         <v/>
       </c>
-      <c r="U51" s="35">
-        <f>K51-T51</f>
-        <v/>
+      <c r="U51" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -6463,14 +6708,21 @@
       </c>
       <c r="M52" s="31" t="n">
         <v>206387500</v>
+      </c>
+      <c r="N52" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O52" s="4" t="n">
+        <v>1876250000</v>
       </c>
       <c r="T52" s="36">
         <f>O52+Q52+S52</f>
         <v/>
       </c>
-      <c r="U52" s="35">
-        <f>K52-T52</f>
-        <v/>
+      <c r="U52" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -6517,14 +6769,21 @@
       </c>
       <c r="M53" s="31" t="n">
         <v>212905000</v>
+      </c>
+      <c r="N53" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O53" s="4" t="n">
+        <v>1935500000</v>
       </c>
       <c r="T53" s="36">
         <f>O53+Q53+S53</f>
         <v/>
       </c>
-      <c r="U53" s="35">
-        <f>K53-T53</f>
-        <v/>
+      <c r="U53" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -6571,14 +6830,21 @@
       </c>
       <c r="M54" s="31" t="n">
         <v>119487500</v>
+      </c>
+      <c r="N54" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O54" s="4" t="n">
+        <v>1086250000</v>
       </c>
       <c r="T54" s="36">
         <f>O54+Q54+S54</f>
         <v/>
       </c>
-      <c r="U54" s="35">
-        <f>K54-T54</f>
-        <v/>
+      <c r="U54" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -6625,14 +6891,21 @@
       </c>
       <c r="M55" s="31" t="n">
         <v>543125000</v>
+      </c>
+      <c r="N55" s="6" t="n">
+        <v>9875000</v>
+      </c>
+      <c r="O55" s="4" t="n">
+        <v>4937500000</v>
       </c>
       <c r="T55" s="36">
         <f>O55+Q55+S55</f>
         <v/>
       </c>
-      <c r="U55" s="35">
-        <f>K55-T55</f>
-        <v/>
+      <c r="U55" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="56">

</xml_diff>

<commit_message>
Implement Math-Match Verification for 100% Qty accuracy, Full Batch Debug Logs, and Auto-Fit Excel columns
</commit_message>
<xml_diff>
--- a/MONITORING PK-PM 31 PUPUK 2026.xlsx
+++ b/MONITORING PK-PM 31 PUPUK 2026.xlsx
@@ -76,7 +76,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -168,15 +168,6 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3658,20 +3649,19 @@
       <c r="M2" s="31" t="n">
         <v>217503000</v>
       </c>
-      <c r="N2" s="38" t="n">
-        <v>6591000</v>
-      </c>
-      <c r="O2" s="39" t="n">
+      <c r="N2" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="O2" s="16" t="n">
         <v>1977300000</v>
       </c>
       <c r="T2" s="36">
         <f>O2+Q2+S2</f>
         <v/>
       </c>
-      <c r="U2" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U2" s="35">
+        <f>K2-T2</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -3719,20 +3709,19 @@
       <c r="M3" s="31" t="n">
         <v>2530000</v>
       </c>
-      <c r="R3" s="38" t="n">
-        <v>575</v>
-      </c>
-      <c r="S3" s="39" t="n">
+      <c r="R3" s="16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="S3" s="16" t="n">
         <v>23000000</v>
       </c>
       <c r="T3" s="36">
         <f>O3+Q3+S3</f>
         <v/>
       </c>
-      <c r="U3" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U3" s="35">
+        <f>K3-T3</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -3780,20 +3769,19 @@
       <c r="M4" s="31" t="n">
         <v>2403500</v>
       </c>
-      <c r="R4" s="38" t="n">
-        <v>575</v>
-      </c>
-      <c r="S4" s="39" t="n">
+      <c r="R4" s="16" t="n">
+        <v>38000</v>
+      </c>
+      <c r="S4" s="16" t="n">
         <v>21850000</v>
       </c>
       <c r="T4" s="36">
         <f>O4+Q4+S4</f>
         <v/>
       </c>
-      <c r="U4" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U4" s="35">
+        <f>K4-T4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -3841,20 +3829,19 @@
       <c r="M5" s="31" t="n">
         <v>570900</v>
       </c>
-      <c r="R5" s="38" t="n">
-        <v>173</v>
-      </c>
-      <c r="S5" s="39" t="n">
+      <c r="R5" s="16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="S5" s="16" t="n">
         <v>5190000</v>
       </c>
       <c r="T5" s="36">
         <f>O5+Q5+S5</f>
         <v/>
       </c>
-      <c r="U5" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U5" s="35">
+        <f>K5-T5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -3902,20 +3889,19 @@
       <c r="M6" s="31" t="n">
         <v>14219865</v>
       </c>
-      <c r="R6" s="38" t="n">
-        <v>3450</v>
-      </c>
-      <c r="S6" s="39" t="n">
+      <c r="R6" s="16" t="n">
+        <v>224820</v>
+      </c>
+      <c r="S6" s="16" t="n">
         <v>129271500</v>
       </c>
       <c r="T6" s="36">
         <f>O6+Q6+S6</f>
         <v/>
       </c>
-      <c r="U6" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U6" s="35">
+        <f>K6-T6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -3968,20 +3954,19 @@
       <c r="M7" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N7" s="38" t="n">
-        <v>6591000</v>
-      </c>
-      <c r="O7" s="39" t="n">
+      <c r="N7" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="O7" s="16" t="n">
         <v>1318200000</v>
       </c>
       <c r="T7" s="36">
         <f>O7+Q7+S7</f>
         <v/>
       </c>
-      <c r="U7" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U7" s="35">
+        <f>K7-T7</f>
+        <v/>
       </c>
     </row>
     <row r="8" hidden="1">
@@ -4094,8 +4079,8 @@
       <c r="M9" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N9" s="38" t="n">
-        <v>6591000</v>
+      <c r="N9" s="16" t="n">
+        <v>200</v>
       </c>
       <c r="O9" s="13" t="n">
         <v>1318200000</v>
@@ -4104,10 +4089,9 @@
         <f>O9+Q9+S9</f>
         <v/>
       </c>
-      <c r="U9" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U9" s="35">
+        <f>K9-T9</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -4155,8 +4139,8 @@
       <c r="M10" s="31" t="n">
         <v>4680500</v>
       </c>
-      <c r="R10" s="38" t="n">
-        <v>1150</v>
+      <c r="R10" s="16" t="n">
+        <v>74000</v>
       </c>
       <c r="S10" s="13" t="n">
         <v>42550000</v>
@@ -4165,10 +4149,9 @@
         <f>O10+Q10+S10</f>
         <v/>
       </c>
-      <c r="U10" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U10" s="35">
+        <f>K10-T10</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -4216,8 +4199,8 @@
       <c r="M11" s="31" t="n">
         <v>12650000</v>
       </c>
-      <c r="R11" s="38" t="n">
-        <v>2875</v>
+      <c r="R11" s="16" t="n">
+        <v>200000</v>
       </c>
       <c r="S11" s="13" t="n">
         <v>115000000</v>
@@ -4226,10 +4209,9 @@
         <f>O11+Q11+S11</f>
         <v/>
       </c>
-      <c r="U11" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U11" s="35">
+        <f>K11-T11</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -4277,8 +4259,8 @@
       <c r="M12" s="31" t="n">
         <v>9297750</v>
       </c>
-      <c r="R12" s="38" t="n">
-        <v>2300</v>
+      <c r="R12" s="16" t="n">
+        <v>147000</v>
       </c>
       <c r="S12" s="13" t="n">
         <v>84525000</v>
@@ -4287,10 +4269,9 @@
         <f>O12+Q12+S12</f>
         <v/>
       </c>
-      <c r="U12" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U12" s="35">
+        <f>K12-T12</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -4343,22 +4324,19 @@
       <c r="M13" s="31" t="n">
         <v>18150000</v>
       </c>
-      <c r="P13" s="6" t="n">
-        <v>550</v>
-      </c>
-      <c r="Q13" s="4" t="n">
+      <c r="R13" s="16" t="n">
+        <v>300000</v>
+      </c>
+      <c r="S13" s="13" t="n">
         <v>165000000</v>
       </c>
-      <c r="R13" s="16" t="n"/>
-      <c r="S13" s="13" t="n"/>
       <c r="T13" s="36">
         <f>O13+Q13+S13</f>
         <v/>
       </c>
-      <c r="U13" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U13" s="35">
+        <f>K13-T13</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -4406,8 +4384,8 @@
       <c r="M14" s="31" t="n">
         <v>8855000</v>
       </c>
-      <c r="R14" s="38" t="n">
-        <v>575</v>
+      <c r="R14" s="16" t="n">
+        <v>140000</v>
       </c>
       <c r="S14" s="13" t="n">
         <v>80500000</v>
@@ -4416,10 +4394,9 @@
         <f>O14+Q14+S14</f>
         <v/>
       </c>
-      <c r="U14" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U14" s="35">
+        <f>K14-T14</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -4472,8 +4449,8 @@
       <c r="M15" s="31" t="n">
         <v>77858000</v>
       </c>
-      <c r="N15" s="38" t="n">
-        <v>7078000</v>
+      <c r="N15" s="16" t="n">
+        <v>100</v>
       </c>
       <c r="O15" s="13" t="n">
         <v>707800000</v>
@@ -4482,10 +4459,9 @@
         <f>O15+Q15+S15</f>
         <v/>
       </c>
-      <c r="U15" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U15" s="35">
+        <f>K15-T15</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -4538,8 +4514,8 @@
       <c r="M16" s="31" t="n">
         <v>145002000</v>
       </c>
-      <c r="N16" s="38" t="n">
-        <v>6591000</v>
+      <c r="N16" s="16" t="n">
+        <v>200</v>
       </c>
       <c r="O16" s="13" t="n">
         <v>1318200000</v>
@@ -4548,10 +4524,9 @@
         <f>O16+Q16+S16</f>
         <v/>
       </c>
-      <c r="U16" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U16" s="35">
+        <f>K16-T16</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -4604,12 +4579,14 @@
       <c r="M17" s="31" t="n">
         <v>1960750</v>
       </c>
-      <c r="R17" s="38" t="n">
+      <c r="P17" s="6" t="n">
         <v>575</v>
       </c>
-      <c r="S17" s="39" t="n">
+      <c r="Q17" s="4" t="n">
         <v>17825000</v>
       </c>
+      <c r="R17" s="16" t="n"/>
+      <c r="S17" s="16" t="n"/>
       <c r="T17" s="36">
         <f>O17+Q17+S17</f>
         <v/>
@@ -4670,20 +4647,20 @@
       <c r="M18" s="31" t="n">
         <v>3921500</v>
       </c>
-      <c r="R18" s="38" t="n">
-        <v>1150</v>
-      </c>
-      <c r="S18" s="39" t="n">
+      <c r="R18" s="16">
+        <f>31000+31000</f>
+        <v/>
+      </c>
+      <c r="S18" s="16" t="n">
         <v>35650000</v>
       </c>
       <c r="T18" s="36">
         <f>O18+Q18+S18</f>
         <v/>
       </c>
-      <c r="U18" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U18" s="35">
+        <f>K18-T18</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -4731,20 +4708,19 @@
       <c r="M19" s="31" t="n">
         <v>13768480</v>
       </c>
-      <c r="R19" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="S19" s="39" t="n">
+      <c r="R19" s="16" t="n">
+        <v>782300</v>
+      </c>
+      <c r="S19" s="16" t="n">
         <v>125168000</v>
       </c>
       <c r="T19" s="36">
         <f>O19+Q19+S19</f>
         <v/>
       </c>
-      <c r="U19" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U19" s="35">
+        <f>K19-T19</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -4797,20 +4773,19 @@
       <c r="M20" s="31" t="n">
         <v>2277000</v>
       </c>
-      <c r="R20" s="38" t="n">
-        <v>575</v>
-      </c>
-      <c r="S20" s="39" t="n">
+      <c r="R20" s="16" t="n">
+        <v>36000</v>
+      </c>
+      <c r="S20" s="16" t="n">
         <v>20700000</v>
       </c>
       <c r="T20" s="36">
         <f>O20+Q20+S20</f>
         <v/>
       </c>
-      <c r="U20" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U20" s="35">
+        <f>K20-T20</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -4860,8 +4835,12 @@
       </c>
       <c r="N21" s="16" t="n"/>
       <c r="O21" s="16" t="n"/>
-      <c r="P21" s="16" t="n"/>
-      <c r="Q21" s="16" t="n"/>
+      <c r="P21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="16" t="n">
+        <v>16250000</v>
+      </c>
       <c r="R21" s="16" t="n"/>
       <c r="S21" s="16" t="n"/>
       <c r="T21" s="36">
@@ -4932,20 +4911,19 @@
       <c r="O22" s="16" t="n"/>
       <c r="P22" s="16" t="n"/>
       <c r="Q22" s="16" t="n"/>
-      <c r="R22" s="38" t="n">
-        <v>170</v>
-      </c>
-      <c r="S22" s="39" t="n">
+      <c r="R22" s="16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="S22" s="16" t="n">
         <v>5100000</v>
       </c>
       <c r="T22" s="36">
         <f>O22+Q22+S22</f>
         <v/>
       </c>
-      <c r="U22" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U22" s="35">
+        <f>K22-T22</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -5002,8 +4980,8 @@
       <c r="O23" s="16" t="n"/>
       <c r="P23" s="16" t="n"/>
       <c r="Q23" s="16" t="n"/>
-      <c r="R23" s="38" t="n">
-        <v>580</v>
+      <c r="R23" s="16" t="n">
+        <v>179758</v>
       </c>
       <c r="S23" s="18" t="n">
         <v>104259640</v>
@@ -5012,10 +4990,9 @@
         <f>O23+Q23+S23</f>
         <v/>
       </c>
-      <c r="U23" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U23" s="35">
+        <f>K23-T23</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -5072,8 +5049,8 @@
       <c r="O24" s="16" t="n"/>
       <c r="P24" s="16" t="n"/>
       <c r="Q24" s="16" t="n"/>
-      <c r="R24" s="38" t="n">
-        <v>575</v>
+      <c r="R24" s="16" t="n">
+        <v>27000</v>
       </c>
       <c r="S24" s="18" t="n">
         <v>15525000</v>
@@ -5082,10 +5059,9 @@
         <f>O24+Q24+S24</f>
         <v/>
       </c>
-      <c r="U24" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U24" s="35">
+        <f>K24-T24</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -5133,20 +5109,19 @@
       <c r="M25" s="31" t="n">
         <v>2332000</v>
       </c>
-      <c r="R25" s="38" t="n">
-        <v>530</v>
-      </c>
-      <c r="S25" s="39" t="n">
+      <c r="R25" s="16" t="n">
+        <v>120000</v>
+      </c>
+      <c r="S25" s="16" t="n">
         <v>21200000</v>
       </c>
       <c r="T25" s="36">
         <f>O25+Q25+S25</f>
         <v/>
       </c>
-      <c r="U25" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U25" s="35">
+        <f>K25-T25</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -5194,20 +5169,19 @@
       <c r="M26" s="31" t="n">
         <v>3520000</v>
       </c>
-      <c r="R26" s="38" t="n">
-        <v>800</v>
-      </c>
-      <c r="S26" s="39" t="n">
+      <c r="R26" s="16" t="n">
+        <v>200000</v>
+      </c>
+      <c r="S26" s="16" t="n">
         <v>32000000</v>
       </c>
       <c r="T26" s="36">
         <f>O26+Q26+S26</f>
         <v/>
       </c>
-      <c r="U26" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U26" s="35">
+        <f>K26-T26</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -5255,20 +5229,19 @@
       <c r="M27" s="31" t="n">
         <v>704000</v>
       </c>
-      <c r="R27" s="38" t="n">
-        <v>160</v>
-      </c>
-      <c r="S27" s="39" t="n">
+      <c r="R27" s="16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="S27" s="16" t="n">
         <v>6400000</v>
       </c>
       <c r="T27" s="36">
         <f>O27+Q27+S27</f>
         <v/>
       </c>
-      <c r="U27" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U27" s="35">
+        <f>K27-T27</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -5321,10 +5294,10 @@
       <c r="M28" s="31" t="n">
         <v>696963960</v>
       </c>
-      <c r="N28" s="38" t="n">
-        <v>6426000</v>
-      </c>
-      <c r="O28" s="39" t="n">
+      <c r="N28" s="16" t="n">
+        <v>986</v>
+      </c>
+      <c r="O28" s="16" t="n">
         <v>6336036000</v>
       </c>
       <c r="P28" s="16" t="n"/>
@@ -5335,10 +5308,9 @@
         <f>O28+Q28+S28</f>
         <v/>
       </c>
-      <c r="U28" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U28" s="35">
+        <f>K28-T28</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -5391,8 +5363,8 @@
       <c r="M29" s="31" t="n">
         <v>159043500</v>
       </c>
-      <c r="N29" s="38" t="n">
-        <v>6426000</v>
+      <c r="N29" s="16" t="n">
+        <v>225</v>
       </c>
       <c r="O29" s="13" t="n">
         <v>1445850000</v>
@@ -5405,10 +5377,9 @@
         <f>O29+Q29+S29</f>
         <v/>
       </c>
-      <c r="U29" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U29" s="35">
+        <f>K29-T29</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -5460,8 +5431,8 @@
       <c r="O30" s="16" t="n"/>
       <c r="P30" s="16" t="n"/>
       <c r="Q30" s="16" t="n"/>
-      <c r="R30" s="38" t="n">
-        <v>640</v>
+      <c r="R30" s="16" t="n">
+        <v>160000</v>
       </c>
       <c r="S30" s="18" t="n">
         <v>25600000</v>
@@ -5470,10 +5441,9 @@
         <f>O30+Q30+S30</f>
         <v/>
       </c>
-      <c r="U30" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U30" s="35">
+        <f>K30-T30</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -5526,8 +5496,8 @@
       <c r="M31" s="31" t="n">
         <v>473660000</v>
       </c>
-      <c r="N31" s="38" t="n">
-        <v>8612000</v>
+      <c r="N31" s="16" t="n">
+        <v>500</v>
       </c>
       <c r="O31" s="13" t="n">
         <v>4306000000</v>
@@ -5540,10 +5510,9 @@
         <f>O31+Q31+S31</f>
         <v/>
       </c>
-      <c r="U31" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U31" s="35">
+        <f>K31-T31</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -5593,8 +5562,12 @@
       </c>
       <c r="N32" s="16" t="n"/>
       <c r="O32" s="16" t="n"/>
-      <c r="P32" s="16" t="n"/>
-      <c r="Q32" s="18" t="n"/>
+      <c r="P32" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="18" t="n">
+        <v>16250000</v>
+      </c>
       <c r="R32" s="16" t="n"/>
       <c r="S32" s="16" t="n"/>
       <c r="T32" s="36">
@@ -5651,20 +5624,19 @@
       <c r="M33" s="31" t="n">
         <v>1408000</v>
       </c>
-      <c r="R33" s="38" t="n">
-        <v>320</v>
-      </c>
-      <c r="S33" s="39" t="n">
+      <c r="R33" s="16" t="n">
+        <v>80000</v>
+      </c>
+      <c r="S33" s="16" t="n">
         <v>12800000</v>
       </c>
       <c r="T33" s="36">
         <f>O33+Q33+S33</f>
         <v/>
       </c>
-      <c r="U33" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U33" s="35">
+        <f>K33-T33</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -5712,20 +5684,19 @@
       <c r="M34" s="31" t="n">
         <v>1408000</v>
       </c>
-      <c r="R34" s="38" t="n">
-        <v>320</v>
-      </c>
-      <c r="S34" s="39" t="n">
+      <c r="R34" s="16" t="n">
+        <v>80000</v>
+      </c>
+      <c r="S34" s="16" t="n">
         <v>12800000</v>
       </c>
       <c r="T34" s="36">
         <f>O34+Q34+S34</f>
         <v/>
       </c>
-      <c r="U34" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U34" s="35">
+        <f>K34-T34</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -5773,8 +5744,8 @@
       <c r="M35" s="31" t="n">
         <v>2662000</v>
       </c>
-      <c r="R35" s="38" t="n">
-        <v>605</v>
+      <c r="R35" s="16" t="n">
+        <v>120000</v>
       </c>
       <c r="S35" s="13" t="n">
         <v>24200000</v>
@@ -5783,10 +5754,9 @@
         <f>O35+Q35+S35</f>
         <v/>
       </c>
-      <c r="U35" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U35" s="35">
+        <f>K35-T35</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -5834,8 +5804,8 @@
       <c r="M36" s="31" t="n">
         <v>91245000</v>
       </c>
-      <c r="N36" s="40" t="n">
-        <v>9875000</v>
+      <c r="N36" s="14" t="n">
+        <v>84</v>
       </c>
       <c r="O36" s="13" t="n">
         <v>829500000</v>
@@ -5844,10 +5814,9 @@
         <f>O36+Q36+S36</f>
         <v/>
       </c>
-      <c r="U36" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U36" s="35">
+        <f>K36-T36</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -5895,8 +5864,8 @@
       <c r="M37" s="31" t="n">
         <v>94503750</v>
       </c>
-      <c r="N37" s="40" t="n">
-        <v>9875000</v>
+      <c r="N37" s="14" t="n">
+        <v>87</v>
       </c>
       <c r="O37" s="13" t="n">
         <v>859125000</v>
@@ -5905,10 +5874,9 @@
         <f>O37+Q37+S37</f>
         <v/>
       </c>
-      <c r="U37" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U37" s="35">
+        <f>K37-T37</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -5956,8 +5924,8 @@
       <c r="M38" s="31" t="n">
         <v>2552000</v>
       </c>
-      <c r="R38" s="38" t="n">
-        <v>580</v>
+      <c r="R38" s="16" t="n">
+        <v>120</v>
       </c>
       <c r="S38" s="18" t="n">
         <v>23200000</v>
@@ -5966,10 +5934,9 @@
         <f>O38+Q38+S38</f>
         <v/>
       </c>
-      <c r="U38" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U38" s="35">
+        <f>K38-T38</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -6017,20 +5984,19 @@
       <c r="M39" s="31" t="n">
         <v>2937297</v>
       </c>
-      <c r="R39" s="38" t="n">
-        <v>117117.12</v>
+      <c r="R39" s="16" t="n">
+        <v>228</v>
       </c>
       <c r="S39" s="18" t="n">
-        <v>26702703.36</v>
+        <v>26702703</v>
       </c>
       <c r="T39" s="36">
         <f>O39+Q39+S39</f>
         <v/>
       </c>
-      <c r="U39" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U39" s="35">
+        <f>K39-T39</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -6078,10 +6044,10 @@
       <c r="M40" s="31" t="n">
         <v>543125000</v>
       </c>
-      <c r="N40" s="38" t="n">
-        <v>9875000</v>
-      </c>
-      <c r="O40" s="39" t="n">
+      <c r="N40" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="O40" s="16" t="n">
         <v>4937500000</v>
       </c>
       <c r="P40" s="16" t="n"/>
@@ -6092,10 +6058,9 @@
         <f>O40+Q40+S40</f>
         <v/>
       </c>
-      <c r="U40" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U40" s="35">
+        <f>K40-T40</f>
+        <v/>
       </c>
     </row>
     <row r="41" hidden="1">
@@ -6163,8 +6128,8 @@
       <c r="M43" s="31" t="n">
         <v>2442000</v>
       </c>
-      <c r="R43" s="38" t="n">
-        <v>555</v>
+      <c r="R43" s="16" t="n">
+        <v>120000</v>
       </c>
       <c r="S43" s="18" t="n">
         <v>22200000</v>
@@ -6173,10 +6138,9 @@
         <f>O43+Q43+S43</f>
         <v/>
       </c>
-      <c r="U43" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U43" s="35">
+        <f>K43-T43</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -6224,8 +6188,8 @@
       <c r="M44" s="31" t="n">
         <v>3256000</v>
       </c>
-      <c r="R44" s="38" t="n">
-        <v>740</v>
+      <c r="R44" s="16" t="n">
+        <v>160000</v>
       </c>
       <c r="S44" s="18" t="n">
         <v>29600000</v>
@@ -6234,10 +6198,9 @@
         <f>O44+Q44+S44</f>
         <v/>
       </c>
-      <c r="U44" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U44" s="35">
+        <f>K44-T44</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -6285,8 +6248,8 @@
       <c r="M45" s="31" t="n">
         <v>814000</v>
       </c>
-      <c r="R45" s="38" t="n">
-        <v>185</v>
+      <c r="R45" s="16" t="n">
+        <v>40000</v>
       </c>
       <c r="S45" s="18" t="n">
         <v>7400000</v>
@@ -6295,10 +6258,9 @@
         <f>O45+Q45+S45</f>
         <v/>
       </c>
-      <c r="U45" s="35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U45" s="35">
+        <f>K45-T45</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -6347,7 +6309,7 @@
         <v>238975000</v>
       </c>
       <c r="N46" s="6" t="n">
-        <v>9875000</v>
+        <v>220</v>
       </c>
       <c r="O46" s="4" t="n">
         <v>2172500000</v>
@@ -6407,7 +6369,7 @@
         <v>22811250</v>
       </c>
       <c r="N47" s="6" t="n">
-        <v>9875000</v>
+        <v>21</v>
       </c>
       <c r="O47" s="4" t="n">
         <v>207375000</v>
@@ -6467,7 +6429,7 @@
         <v>41277500</v>
       </c>
       <c r="N48" s="6" t="n">
-        <v>9875000</v>
+        <v>38</v>
       </c>
       <c r="O48" s="4" t="n">
         <v>375250000</v>
@@ -6528,7 +6490,7 @@
         <v>41277500</v>
       </c>
       <c r="N49" s="6" t="n">
-        <v>9875000</v>
+        <v>38</v>
       </c>
       <c r="O49" s="4" t="n">
         <v>375250000</v>
@@ -6588,7 +6550,7 @@
         <v>256355000</v>
       </c>
       <c r="N50" s="6" t="n">
-        <v>9875000</v>
+        <v>236</v>
       </c>
       <c r="O50" s="4" t="n">
         <v>2330500000</v>
@@ -6649,7 +6611,7 @@
         <v>304150000</v>
       </c>
       <c r="N51" s="6" t="n">
-        <v>9875000</v>
+        <v>280</v>
       </c>
       <c r="O51" s="4" t="n">
         <v>2765000000</v>
@@ -6710,7 +6672,7 @@
         <v>206387500</v>
       </c>
       <c r="N52" s="6" t="n">
-        <v>9875000</v>
+        <v>190</v>
       </c>
       <c r="O52" s="4" t="n">
         <v>1876250000</v>
@@ -6771,7 +6733,7 @@
         <v>212905000</v>
       </c>
       <c r="N53" s="6" t="n">
-        <v>9875000</v>
+        <v>196</v>
       </c>
       <c r="O53" s="4" t="n">
         <v>1935500000</v>
@@ -6832,7 +6794,7 @@
         <v>119487500</v>
       </c>
       <c r="N54" s="6" t="n">
-        <v>9875000</v>
+        <v>110</v>
       </c>
       <c r="O54" s="4" t="n">
         <v>1086250000</v>
@@ -6893,7 +6855,7 @@
         <v>543125000</v>
       </c>
       <c r="N55" s="6" t="n">
-        <v>9875000</v>
+        <v>500</v>
       </c>
       <c r="O55" s="4" t="n">
         <v>4937500000</v>

</xml_diff>